<commit_message>
Removed excel file reading and implemented scenario outline
</commit_message>
<xml_diff>
--- a/DEMOWEBSHOP/src/test/resources/TestData/wishlistData.xlsx
+++ b/DEMOWEBSHOP/src/test/resources/TestData/wishlistData.xlsx
@@ -8,12 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DWS\AUTOMATIONPROJECT\DEMOWEBSHOP\src\test\resources\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{3A3B0D7F-07EB-4CE1-8A1B-0A96FE36C8B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CD6D8A9-C6F9-4B0D-9FF5-A5D85559E854}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA2B9002-DEE5-4151-849E-4D61E4DD6FF8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{AA2B9002-DEE5-4151-849E-4D61E4DD6FF8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="AddWishlist" sheetId="1" r:id="rId1"/>
+    <sheet name="RemoveWishlist" sheetId="2" r:id="rId2"/>
+    <sheet name="DisplayWishlist" sheetId="3" r:id="rId3"/>
+    <sheet name="WishlistToCart" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,10 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
-  <si>
-    <t>scenario</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="12">
   <si>
     <t>product</t>
   </si>
@@ -47,31 +47,34 @@
     <t>expectedMessage</t>
   </si>
   <si>
-    <t>AddWishlist</t>
-  </si>
-  <si>
     <t>Health Book</t>
   </si>
   <si>
     <t>The product has been added to your wishlist</t>
   </si>
   <si>
-    <t>RemoveWishlist</t>
-  </si>
-  <si>
     <t>Fiction EX</t>
   </si>
   <si>
-    <t>WishlistToCart</t>
-  </si>
-  <si>
     <t>Smartphone</t>
   </si>
   <si>
-    <t>DisplayWishlist</t>
-  </si>
-  <si>
-    <t>Black &amp; White Diamond Heart</t>
+    <t>Laptop</t>
+  </si>
+  <si>
+    <t>Headphones</t>
+  </si>
+  <si>
+    <t>Tablet</t>
+  </si>
+  <si>
+    <t>Camera</t>
+  </si>
+  <si>
+    <t>Keyboard</t>
+  </si>
+  <si>
+    <t>The wishlist is empty</t>
   </si>
 </sst>
 </file>
@@ -457,62 +460,229 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86DF8830-7723-45C1-B325-609DD6BAA52A}">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="22.6640625" customWidth="1"/>
+    <col min="2" max="2" width="29.6640625" customWidth="1"/>
+    <col min="3" max="3" width="60.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1"/>
+    </row>
+    <row r="2" spans="1:3" ht="22.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D8D8BE2-70DA-4D75-9596-0445BFF2FAD5}">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="21.44140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="30.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" ht="33" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C8598B8-A262-438B-AD99-3EB728E55441}">
+  <dimension ref="A1:A6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF001ECA-8701-4848-ACFE-378934751DE4}">
+  <dimension ref="A1:A5"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="2" t="s">
+    <row r="4" spans="1:1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="2" t="s">
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" s="2" t="s">
         <v>8</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="86.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>